<commit_message>
data(matriz): LATAM Pass comision 15% (envio tarifario pendiente)
</commit_message>
<xml_diff>
--- a/data/planillas/matriz_tarifas_canal.xlsx
+++ b/data/planillas/matriz_tarifas_canal.xlsx
@@ -5373,7 +5373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>logística BlueX/Recíbelo pendiente</t>
+          <t>logística = tarifario BlueX/Recíbelo (pendiente rate card)</t>
         </is>
       </c>
     </row>
@@ -5431,6 +5431,24 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>logística pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LATAM Pass</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>15</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>comisión 15%; envío = tarifario BlueX/Recíbelo (pendiente)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(matriz): comisiones B2B 3.4%, webs (UnionX/Lhotse/Simplit) 3%, GRS 0
</commit_message>
<xml_diff>
--- a/data/planillas/matriz_tarifas_canal.xlsx
+++ b/data/planillas/matriz_tarifas_canal.xlsx
@@ -5373,7 +5373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>logística = tarifario BlueX/Recíbelo (pendiente rate card)</t>
+          <t>envío = tarifario BlueX/Recíbelo (por comuna×peso)</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5430,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>logística pendiente</t>
+          <t>envío pendiente</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,97 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>comisión 15%; envío = tarifario BlueX/Recíbelo (pendiente)</t>
+          <t>comisión 15%; envío tarifario</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UnionX B2B</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>comisión 3.4%; envío tarifario</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>UnionX web</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cliente Shopify 3%; envío tarifario</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lhotse web</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>cliente Shopify 3%; envío tarifario</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Simplit web</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cliente Shopify 3%; envío tarifario</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Global Reward</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sin comisión; solo envío tarifario</t>
         </is>
       </c>
     </row>

</xml_diff>